<commit_message>
fix(afp): remove default semantic template normalization and refresh governed artifacts
</commit_message>
<xml_diff>
--- a/management/docs/policy-governance-events.xlsx
+++ b/management/docs/policy-governance-events.xlsx
@@ -9,13 +9,13 @@
     <sheet name="Governance Events" r:id="rId3" sheetId="1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">'Governance Events'!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">'Governance Events'!$A$1:$I$10</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="58">
   <si>
     <t>event_id</t>
   </si>
@@ -177,6 +177,18 @@
   </si>
   <si>
     <t>product/afp-converter/afp-cli/build.gradle|build.gradle|management/pm/workflow/sample-output-reference-manifest.json|AI-POLICY.md|README.md|management/docs/project-plan-progress.csv</t>
+  </si>
+  <si>
+    <t>GOV-2026-02-24-003</t>
+  </si>
+  <si>
+    <t>20260224T000000Z-renderer-output-detemplate</t>
+  </si>
+  <si>
+    <t>Resolved renderer normalization regression by enforcing raw AFP text HTML defaults, explicit semantic-template opt-in, and workstream-governed validation across sample corpus.</t>
+  </si>
+  <si>
+    <t>product/afp-converter/afp-engine/src/main/java/solutions/pointzero/symphony/afp/engine/AfpHtmlRenderer.java|product/afp-converter/afp-engine/src/main/java/solutions/pointzero/symphony/afp/engine/FakeEngineOutputGenerator.java|management/docs/project-plan-progress.csv|management/pm/workflow/workstream-realm-map.json</t>
   </si>
 </sst>
 </file>
@@ -221,7 +233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -485,8 +497,37 @@
         <v>17</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="I10" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
+  <autoFilter ref="A1:I10"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>